<commit_message>
Remove SelgerEierKommune and SelgerBrukerFylke from output
Drops from_owner_municipalityName and from_user_countyName (seller's
municipality, and the "user" party's county) from both
ofv_transactions_lookup.py and the VBA module's output, plus the
matching header columns in the prebuilt OFV_Verktoy.xlsx.

Also hardens the VBA macro's Resultat-sheet reset: it now clears the
whole used range (Cells.ClearContents) instead of only the columns in
the current field map, so removing columns like these doesn't leave
stale data sitting in the old columns on a re-run.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AiRciDcmJUFDDcggXD2bbE
</commit_message>
<xml_diff>
--- a/OFV_Verktoy.xlsx
+++ b/OFV_Verktoy.xlsx
@@ -538,9 +538,9 @@
     <col width="16" customWidth="1" min="14" max="14"/>
     <col width="17" customWidth="1" min="15" max="15"/>
     <col width="17" customWidth="1" min="16" max="16"/>
-    <col width="19" customWidth="1" min="17" max="17"/>
-    <col width="19" customWidth="1" min="18" max="18"/>
-    <col width="16" customWidth="1" min="19" max="19"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="17" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
     <col width="17" customWidth="1" min="20" max="20"/>
     <col width="14" customWidth="1" min="21" max="21"/>
   </cols>
@@ -628,29 +628,21 @@
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>SelgerEierKommune</t>
+          <t>KjoperEierType</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>SelgerBrukerFylke</t>
+          <t>KjoperEierFirma</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>KjoperEierType</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>KjoperEierFirma</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
           <t>Status</t>
         </is>
       </c>
+      <c r="T1" s="1" t="n"/>
+      <c r="U1" s="1" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>